<commit_message>
cambio menor a pasos de error absoluto y relativo
</commit_message>
<xml_diff>
--- a/errores_truncamiento.xlsx
+++ b/errores_truncamiento.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,136 +520,6 @@
       </c>
       <c r="H3" t="n">
         <v>0.0075</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>169335.93</v>
-      </c>
-      <c r="C4" t="n">
-        <v>10583.49</v>
-      </c>
-      <c r="D4" t="n">
-        <v>10583.495625</v>
-      </c>
-      <c r="E4" t="n">
-        <v>179919.42</v>
-      </c>
-      <c r="F4" t="n">
-        <v>179919.425625</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.005625</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.013125</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="n">
-        <v>179919.42</v>
-      </c>
-      <c r="C5" t="n">
-        <v>11244.96</v>
-      </c>
-      <c r="D5" t="n">
-        <v>11244.96375</v>
-      </c>
-      <c r="E5" t="n">
-        <v>191164.38</v>
-      </c>
-      <c r="F5" t="n">
-        <v>191164.38375</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.00375</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.016875</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="n">
-        <v>191164.38</v>
-      </c>
-      <c r="C6" t="n">
-        <v>11947.77</v>
-      </c>
-      <c r="D6" t="n">
-        <v>11947.77375</v>
-      </c>
-      <c r="E6" t="n">
-        <v>203112.15</v>
-      </c>
-      <c r="F6" t="n">
-        <v>203112.15375</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.00375</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.020625</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>203112.15</v>
-      </c>
-      <c r="C7" t="n">
-        <v>12694.5</v>
-      </c>
-      <c r="D7" t="n">
-        <v>12694.509375</v>
-      </c>
-      <c r="E7" t="n">
-        <v>215806.65</v>
-      </c>
-      <c r="F7" t="n">
-        <v>215806.659375</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.009375</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="n">
-        <v>215806.65</v>
-      </c>
-      <c r="C8" t="n">
-        <v>13487.91</v>
-      </c>
-      <c r="D8" t="n">
-        <v>13487.915625</v>
-      </c>
-      <c r="E8" t="n">
-        <v>229294.56</v>
-      </c>
-      <c r="F8" t="n">
-        <v>229294.565625</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.005625</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.035625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>